<commit_message>
Jedna aplikacja: scalenie treści raportu, modelu v1 i audytu; deklaracja finansowania; nawigacja w grupach (28.10.2026)
</commit_message>
<xml_diff>
--- a/pobierz/hcv_model_inwestycji.xlsx
+++ b/pobierz/hcv_model_inwestycji.xlsx
@@ -21,7 +21,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodologia" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Na_pacjenta" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analizy_scen" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zmiany" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leki_zamowienia" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zmiany" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="x_N0">Parametry!$C$2</definedName>
@@ -562,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -642,6 +643,13 @@
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Materiał edukacyjny, neutralny; bez nazw leków i firm. Recenzja panelu ról w aplikacji jest symulowana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Deklaracja finansowania i konfliktu interesów: Autor pracuje w sektorze farmaceutycznym. Analiza powstała prywatnie, bez zlecenia i finansowania jakiejkolwiek firmy. Nie wymienia ani nie promuje żadnych produktów leczniczych. Część wykorzystanych źródeł była finansowana przez przemysł — oznaczono to w Źródłach.</t>
         </is>
       </c>
     </row>
@@ -13437,7 +13445,254 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Leki i zamówienia publiczne – dane źródłowe (nie wyniki modelu); schematy bez nazw leków i firm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Schemat B.71, 2025</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Pacjenci</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Refundacja (mln zł)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Uwagi / źródło</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>A – pangenotypowy</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2398</v>
+      </c>
+      <c r="C4" t="n">
+        <v>55.46</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NFZ app-stat-api, pobrane 25.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B – pangenotypowy</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2396</v>
+      </c>
+      <c r="C5" t="n">
+        <v>52.53</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>zmiana ceny urzędowej 17.09.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C – leczenie ponowne</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>61</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>zmiana ceny urzędowej 17.06.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B.71 razem (leczeni, nie suma schematów)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4832</v>
+      </c>
+      <c r="C7" t="n">
+        <v>109.98</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>NFZ app-stat-api, pobrane 25.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Przetargi TED od 01.01.2023 (pobrane 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ogłoszenia</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Części z wyborem oferty</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Wartość (mln zł)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>229</v>
+      </c>
+      <c r="C10" t="n">
+        <v>61</v>
+      </c>
+      <c r="D10" t="n">
+        <v>88.53</v>
+      </c>
+      <c r="E10" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="F10" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="G10" t="n">
+        <v>22.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>289</v>
+      </c>
+      <c r="C11" t="n">
+        <v>66</v>
+      </c>
+      <c r="D11" t="n">
+        <v>81.36</v>
+      </c>
+      <c r="E11" t="n">
+        <v>29</v>
+      </c>
+      <c r="F11" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="G11" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>177</v>
+      </c>
+      <c r="C12" t="n">
+        <v>43</v>
+      </c>
+      <c r="D12" t="n">
+        <v>13.83</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Razem bez podwójnego liczenia (7 części mieszanych, 6,68 mln zł)</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Uwaga: TED obejmuje tylko przetargi powyżej progów UE; wartość przetargu ≠ sprzedaż. 38 zamawiających; 10 największych ≈123,6 mln zł (≈70%).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -13552,6 +13807,20 @@
       <c r="A16" t="inlineStr">
         <is>
           <t>Dodatkowo: w pliku xlsx usunięto kolizję nazw zakresów (stopa dyskonta kosztów i efektów) – po poprawce wartości w arkuszu zgadzają się ze stroną.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Deklaracja finansowania i konfliktu interesów (28.10.2026, CHEERS 2022): Autor pracuje w sektorze farmaceutycznym. Analiza powstała prywatnie, bez zlecenia i finansowania jakiejkolwiek firmy. Nie wymienia ani nie promuje żadnych produktów leczniczych. Część wykorzystanych źródeł była finansowana przez przemysł — oznaczono to w Źródłach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Jedna aplikacja (28.10.2026): do aplikacji przeniesiono całą wartościową treść wcześniejszych roboczych stron raportu, modelu v1 i audytu – hipotezy H1–H6 (Problem), nowa zakładka „Leki i zamówienia publiczne” (schematy B.71 bez nazw, przetargi TED), ocena działań systemowych A1–A9 (Działania), przebieg audytu (ocena, odtworzenie, weryfikacja parametrów, wrażliwość), szacunek Polaris liczby leczonych 2015–2023, porównanie zgłaszalności z Litwą, najdłuższe kolejki do B.71 i nowe luki w danych. Nawigacja pogrupowana: Odpowiedź / Problem i rynek / Działania / Metoda i źródła. Treści o charakterze komercyjnym nie zostały przeniesione.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Inwentarz danych: przywrócenie pominiętych danych publicznych z wcześniejszych wersji (źródła, daty); tabela weryfikacji 33 parametrów; ograniczenia
</commit_message>
<xml_diff>
--- a/pobierz/hcv_model_inwestycji.xlsx
+++ b/pobierz/hcv_model_inwestycji.xlsx
@@ -13692,7 +13692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -13821,6 +13821,13 @@
       <c r="A18" t="inlineStr">
         <is>
           <t>Jedna aplikacja (28.10.2026): do aplikacji przeniesiono całą wartościową treść wcześniejszych roboczych stron raportu, modelu v1 i audytu – hipotezy H1–H6 (Problem), nowa zakładka „Leki i zamówienia publiczne” (schematy B.71 bez nazw, przetargi TED), ocena działań systemowych A1–A9 (Działania), przebieg audytu (ocena, odtworzenie, weryfikacja parametrów, wrażliwość), szacunek Polaris liczby leczonych 2015–2023, porównanie zgłaszalności z Litwą, najdłuższe kolejki do B.71 i nowe luki w danych. Nawigacja pogrupowana: Odpowiedź / Problem i rynek / Działania / Metoda i źródła. Treści o charakterze komercyjnym nie zostały przeniesione.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Inwentarz danych (28.10.2026): porównano aplikację ze wszystkimi wcześniejszymi wersjami i przywrócono pominięte dane publiczne – 0,47% z wiremią w badaniu POZ 2012–2016 (PLoS One 2017), trend rozpoznań +23% i leczonych −43% wobec 2019 r., 57% uczestników Moje Zdrowie poniżej 40 lat i ok. +20% rozpoznań po 11 miesiącach programu (MZ, IV 2026), 4 010 osób w leczeniu substytucyjnym (EUDA 2024, dane 2022), 93 339 rozpoczęć leczenia w Anglii 2015–2024 (UKHSA 2026), interpretację luk wojewódzkich, sposób liczenia mediany kolejki (37 z 91 lokalizacji), dodatkowe ograniczenie modelu (opieka nieformalna, pomoc społeczna, PFRON, prezenteizm) oraz pełną tabelę weryfikacji 33 parametrów z audytu. Wyniki modelu bez zmian.</t>
         </is>
       </c>
     </row>

</xml_diff>